<commit_message>
feat(categories): integrate Shopee PH category IDs and nail category mapping
- Add configs/categories/shopee_ph_categories.json (1,339 categories, 5-level hierarchy)
- Add configs/categories/shopee_ph_categories.csv (same data, CSV format)
- Add configs/categories/README.md (data dictionary documentation)
- Add configs/nail_category_ids.yaml: nail product category quick-reference
  - 101615: Base & Top Coat (底胶/封层)
  - 102029: Nail Polish (甲油胶/猫眼胶/功能胶) [default]
  - 102030: Nail Polish Remover (卸甲液)
  - 102031: Nail Treatment (护甲油)
  - 102032: Artificial Nail (假指甲)
  - 102033: Nail Art & Sticker (美甲贴纸)
  - 102034: Manicure Tools & Devices (美甲工具/灯/磁铁)
- Add scripts/find_category.py: keyword search tool for category IDs
- Update fixture category_id: 100350 -> 102029 (correct Nail Polish category)
- Update bigseller_mapping.yaml default category_id to 102029
- Revalidate: 15/15 tests passing
</commit_message>
<xml_diff>
--- a/outputs/HMT-CAT-EYE-001/bigseller_product_upload.xlsx
+++ b/outputs/HMT-CAT-EYE-001/bigseller_product_upload.xlsx
@@ -622,7 +622,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>100350</t>
+          <t>102029</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -741,7 +741,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>100350</t>
+          <t>102029</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -860,7 +860,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>100350</t>
+          <t>102029</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -979,7 +979,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>100350</t>
+          <t>102029</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">

</xml_diff>